<commit_message>
bug fixed in data_process_baidu.ipynb regarding line_name_full uniqueness and added line_uid_k for better line identification.
</commit_message>
<xml_diff>
--- a/cast/movie_net/movie_network_stats.xlsx
+++ b/cast/movie_net/movie_network_stats.xlsx
@@ -10,8 +10,8 @@
     <sheet name="原始数据统计" sheetId="1" r:id="rId1"/>
     <sheet name="整体网络图指标" sheetId="2" r:id="rId2"/>
     <sheet name="最大连通子图指标" sheetId="3" r:id="rId3"/>
-    <sheet name="电影二分图指标" sheetId="4" r:id="rId4"/>
-    <sheet name="电影二分图最大连通子图指标" sheetId="5" r:id="rId5"/>
+    <sheet name="作品二分图指标" sheetId="4" r:id="rId4"/>
+    <sheet name="作品二分图最大连通子图指标" sheetId="5" r:id="rId5"/>
     <sheet name="影人二分图指标" sheetId="6" r:id="rId6"/>
     <sheet name="影人二分图最大连通子图指标" sheetId="7" r:id="rId7"/>
   </sheets>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="163">
   <si>
     <t>指标</t>
   </si>
@@ -34,6 +34,9 @@
     <t>说明</t>
   </si>
   <si>
+    <t>作品数量</t>
+  </si>
+  <si>
     <t>导演数量</t>
   </si>
   <si>
@@ -55,6 +58,9 @@
     <t>评分人数标准</t>
   </si>
   <si>
+    <t>200</t>
+  </si>
+  <si>
     <t>130</t>
   </si>
   <si>
@@ -94,6 +100,9 @@
     <t>4.03</t>
   </si>
   <si>
+    <t>电影/电视剧数量</t>
+  </si>
+  <si>
     <t>导演总数</t>
   </si>
   <si>
@@ -103,16 +112,16 @@
     <t>所有影人（包括导演和演员）的总数</t>
   </si>
   <si>
-    <t>所有电影中的最高评分值</t>
-  </si>
-  <si>
-    <t>所有电影中的最低评分值</t>
-  </si>
-  <si>
-    <t>所有电影评分的平均值</t>
-  </si>
-  <si>
-    <t>为保证数据质量，选取评分人数不少于该标准的电影，两者标准可能不同</t>
+    <t>所有作品中的最高评分值</t>
+  </si>
+  <si>
+    <t>所有作品中的最低评分值</t>
+  </si>
+  <si>
+    <t>所有作品评分的平均值</t>
+  </si>
+  <si>
+    <t>为保证数据质量，选取评分人数不少于该标准的作品，两者标准可能不同</t>
   </si>
   <si>
     <t>节点数</t>
@@ -136,19 +145,19 @@
     <t>影人最大介数中心性节点名称</t>
   </si>
   <si>
-    <t>电影节点数</t>
-  </si>
-  <si>
-    <t>电影最大度</t>
-  </si>
-  <si>
-    <t>电影最大度节点名称</t>
-  </si>
-  <si>
-    <t>电影最大介数中心性</t>
-  </si>
-  <si>
-    <t>电影最大介数中心性节点名称</t>
+    <t>作品节点数</t>
+  </si>
+  <si>
+    <t>作品最大度</t>
+  </si>
+  <si>
+    <t>作品最大度节点名称</t>
+  </si>
+  <si>
+    <t>作品最大介数中心性</t>
+  </si>
+  <si>
+    <t>作品最大介数中心性节点名称</t>
   </si>
   <si>
     <t>密度</t>
@@ -190,9 +199,6 @@
     <t>刘德华</t>
   </si>
   <si>
-    <t>200</t>
-  </si>
-  <si>
     <t>108</t>
   </si>
   <si>
@@ -289,19 +295,19 @@
     <t>具有最大介数中心性的影人姓名</t>
   </si>
   <si>
-    <t>电影类型节点的数量</t>
-  </si>
-  <si>
-    <t>电影节点中最大的度值（度：节点连接的边数，反映合作影人数量）</t>
-  </si>
-  <si>
-    <t>具有最大度值的电影名称</t>
-  </si>
-  <si>
-    <t>电影节点中最大的介数中心性值（介数中心性：衡量节点在网络连通中的关键程度）</t>
-  </si>
-  <si>
-    <t>具有最大介数中心性的电影名称</t>
+    <t>作品类型节点的数量</t>
+  </si>
+  <si>
+    <t>作品节点中最大的度值（度：节点连接的边数，反映合作影人数量）</t>
+  </si>
+  <si>
+    <t>具有最大度值的作品名称</t>
+  </si>
+  <si>
+    <t>作品节点中最大的介数中心性值（介数中心性：衡量节点在网络连通中的关键程度）</t>
+  </si>
+  <si>
+    <t>具有最大介数中心性的作品名称</t>
   </si>
   <si>
     <t>网络的密度，表示实际边数与可能最大边数的比值</t>
@@ -860,7 +866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -882,13 +888,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -896,13 +902,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -910,13 +916,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -924,13 +930,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -938,13 +944,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -952,13 +958,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -966,13 +972,27 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1001,268 +1021,268 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1291,212 +1311,212 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1525,184 +1545,184 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1731,128 +1751,128 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D6" t="s">
         <v>137</v>
-      </c>
-      <c r="C6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D6" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1881,184 +1901,184 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2087,128 +2107,128 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
create a detailed commit message for your changes. Lines starting with '#' will be ignored, and an empty message aborts the commit.
</commit_message>
<xml_diff>
--- a/cast/movie_net/movie_network_stats.xlsx
+++ b/cast/movie_net/movie_network_stats.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="121">
   <si>
     <t>指标</t>
   </si>
@@ -61,10 +61,10 @@
     <t>269</t>
   </si>
   <si>
-    <t>3750</t>
-  </si>
-  <si>
-    <t>4009</t>
+    <t>3749</t>
+  </si>
+  <si>
+    <t>4008</t>
   </si>
   <si>
     <t>8.8</t>
@@ -160,7 +160,7 @@
     <t>最大连通子图边比例</t>
   </si>
   <si>
-    <t>4248</t>
+    <t>4247</t>
   </si>
   <si>
     <t>5854</t>
@@ -172,7 +172,7 @@
     <t>王艺禅</t>
   </si>
   <si>
-    <t>0.045796</t>
+    <t>0.046515</t>
   </si>
   <si>
     <t>太保</t>
@@ -184,7 +184,7 @@
     <t>新闻女王2</t>
   </si>
   <si>
-    <t>0.108349</t>
+    <t>0.108506</t>
   </si>
   <si>
     <t>长安的荔枝</t>
@@ -196,19 +196,19 @@
     <t>否</t>
   </si>
   <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>4128</t>
-  </si>
-  <si>
-    <t>97.18%</t>
-  </si>
-  <si>
-    <t>5763</t>
-  </si>
-  <si>
-    <t>98.45%</t>
+    <t>30</t>
+  </si>
+  <si>
+    <t>4132</t>
+  </si>
+  <si>
+    <t>97.29%</t>
+  </si>
+  <si>
+    <t>5767</t>
+  </si>
+  <si>
+    <t>98.51%</t>
   </si>
   <si>
     <t>网络中节点的总数量</t>
@@ -271,19 +271,19 @@
     <t>直径</t>
   </si>
   <si>
-    <t>3921</t>
-  </si>
-  <si>
-    <t>0.048498</t>
-  </si>
-  <si>
-    <t>207</t>
-  </si>
-  <si>
-    <t>0.114742</t>
-  </si>
-  <si>
-    <t>0.000677</t>
+    <t>3924</t>
+  </si>
+  <si>
+    <t>0.049141</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
+    <t>0.114632</t>
+  </si>
+  <si>
+    <t>0.000676</t>
   </si>
   <si>
     <t>是</t>
@@ -307,27 +307,27 @@
     <t>最大介数中心性节点名称</t>
   </si>
   <si>
+    <t>1746</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>0.073125</t>
+  </si>
+  <si>
+    <t>水饺皇后</t>
+  </si>
+  <si>
+    <t>0.06139</t>
+  </si>
+  <si>
+    <t>87.03%</t>
+  </si>
+  <si>
     <t>1744</t>
   </si>
   <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>0.072266</t>
-  </si>
-  <si>
-    <t>水饺皇后</t>
-  </si>
-  <si>
-    <t>0.06132</t>
-  </si>
-  <si>
-    <t>86.61%</t>
-  </si>
-  <si>
-    <t>1742</t>
-  </si>
-  <si>
     <t>99.89%</t>
   </si>
   <si>
@@ -343,10 +343,10 @@
     <t>具有最大介数中心性的节点名称</t>
   </si>
   <si>
-    <t>0.096524</t>
-  </si>
-  <si>
-    <t>0.081703</t>
+    <t>0.096729</t>
+  </si>
+  <si>
+    <t>0.081011</t>
   </si>
   <si>
     <t>6</t>
@@ -361,22 +361,25 @@
     <t>任洛敏</t>
   </si>
   <si>
-    <t>0.045473</t>
-  </si>
-  <si>
-    <t>0.018245</t>
-  </si>
-  <si>
-    <t>97.8%</t>
-  </si>
-  <si>
-    <t>146425</t>
-  </si>
-  <si>
-    <t>0.047538</t>
-  </si>
-  <si>
-    <t>0.019053</t>
+    <t>0.046045</t>
+  </si>
+  <si>
+    <t>0.018254</t>
+  </si>
+  <si>
+    <t>97.9%</t>
+  </si>
+  <si>
+    <t>146431</t>
+  </si>
+  <si>
+    <t>99.9%</t>
+  </si>
+  <si>
+    <t>0.048038</t>
+  </si>
+  <si>
+    <t>0.019025</t>
   </si>
   <si>
     <t>7</t>
@@ -1697,7 +1700,7 @@
         <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
         <v>81</v>
@@ -1773,7 +1776,7 @@
         <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
         <v>105</v>
@@ -1795,7 +1798,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
         <v>75</v>
@@ -1817,7 +1820,7 @@
         <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
         <v>90</v>

</xml_diff>